<commit_message>
Matricule manuel à 5 chiffres au lieu d'auto-généré
- Changer système d'ID : EMP{user.id} → matricule manuel 5 chiffres
- Ajouter validation HTML (pattern, placeholder, title)
- Ajouter validation serveur : format 5 chiffres + unicité
- Mettre à jour import Excel pour accepter colonne Matricule (col 26)
- Messages d'erreur français : 'Le matricule X est déjà utilisé.'
- Fichier de test mis à jour avec matricules : 10001, 10002, 10003
- Tous les tests réussis
</commit_message>
<xml_diff>
--- a/LISTE_SALARIES_25-26.xlsx
+++ b/LISTE_SALARIES_25-26.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Z4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,11 @@
           <t>Taux PAS</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Matricule</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -646,6 +651,11 @@
       <c r="Y2" t="n">
         <v>10.5</v>
       </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -747,6 +757,11 @@
       <c r="Y3" t="n">
         <v>8</v>
       </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>10002</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -847,6 +862,11 @@
       </c>
       <c r="Y4" t="n">
         <v>5</v>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>10003</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>